<commit_message>
Organizei a planilha de dados coletados da calibração do sensor de condutividade
</commit_message>
<xml_diff>
--- a/Programacoes_Condutividade/Dados_Condutividade_04-03.xlsx
+++ b/Programacoes_Condutividade/Dados_Condutividade_04-03.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ufubr-my.sharepoint.com/personal/geovanna_fernandes727_ufu_br/Documents/Área de Trabalho/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gegam\Repositorio_GIT\Peixebinha\Programacoes_Condutividade\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1424F95F-F237-4AD1-8626-14FED3DCDC81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2A7741E-953C-4496-8558-326D57CED339}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{79D3FB78-A525-4967-9C22-E7CE89BAF13F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="10">
   <si>
     <t>uS</t>
   </si>
@@ -63,6 +63,9 @@
   </si>
   <si>
     <t>4ª Leitura</t>
+  </si>
+  <si>
+    <t>uS solução</t>
   </si>
 </sst>
 </file>
@@ -98,13 +101,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -199,7 +205,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="pt-BR"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -1486,20 +1492,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="4"/>
+      <c r="B1" s="5"/>
       <c r="C1" s="1"/>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="3"/>
+      <c r="E1" s="4"/>
       <c r="F1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>2</v>
+      </c>
+      <c r="H1" t="s">
+        <v>9</v>
       </c>
       <c r="I1" s="1"/>
     </row>
@@ -1523,6 +1532,9 @@
       <c r="G2" s="1">
         <v>225</v>
       </c>
+      <c r="H2" s="3">
+        <v>200</v>
+      </c>
       <c r="I2" s="1"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -1545,6 +1557,9 @@
       <c r="G3" s="1">
         <v>438</v>
       </c>
+      <c r="H3" s="1">
+        <v>400</v>
+      </c>
       <c r="I3" s="1"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -1567,6 +1582,9 @@
       <c r="G4" s="1">
         <v>640</v>
       </c>
+      <c r="H4" s="1">
+        <v>600</v>
+      </c>
       <c r="I4" s="1"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -1589,6 +1607,9 @@
       <c r="G5" s="1">
         <v>835</v>
       </c>
+      <c r="H5" s="1">
+        <v>800</v>
+      </c>
       <c r="I5" s="1"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
@@ -1611,6 +1632,9 @@
       <c r="G6" s="1">
         <v>1037</v>
       </c>
+      <c r="H6" s="1">
+        <v>1000</v>
+      </c>
       <c r="I6" s="1"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -1628,10 +1652,10 @@
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="4"/>
+      <c r="B9" s="5"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
@@ -1682,10 +1706,10 @@
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B17" s="4"/>
+      <c r="B17" s="5"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
@@ -1736,10 +1760,10 @@
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B25" s="4"/>
+      <c r="B25" s="5"/>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">

</xml_diff>